<commit_message>
Rewrite Round-3 PO questions (Simple Flow) as plain scenario stories for Milos
Tab 1 reworded to Picture this / What happens today / What we need you to
decide / everyday A-B-C options, jargon-free. Tab 2 QA mapping unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/PO-Questions-Round3.xlsx
+++ b/build/simple-flow/PO-Questions-Round3.xlsx
@@ -520,11 +520,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -537,7 +537,7 @@
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hi Milos! Thanks for your answers to the earlier rounds - they are all actioned. While finishing our checks we found a few more spots where we need your call on how it should work. No wrong answers - for each one, pick an option (or write your own) in the "Your answer" box.</t>
+          <t>Thanks so much, Milos - just pick one option per row; there are no wrong answers, we just need your preference. Each row tells a quick little story of something happening in the shop, then asks what you'd like the app to do.</t>
         </is>
       </c>
     </row>
@@ -549,22 +549,22 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Topic</t>
+          <t>Picture this</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>What happens now</t>
+          <t>What happens today</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>The question</t>
+          <t>What we need you to decide</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Options</t>
+          <t>Your options</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -573,164 +573,167 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="165" customHeight="1">
+    <row r="5" ht="150" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Should a work order have to be reviewed before it can be billed?</t>
+          <t>A mechanic just finished fixing a customer's car, so the repair job is done. Right away, the shop can send the customer their bill - even though nobody has double-checked the mechanic's work yet.</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>When the "needs a review before it is finished" option is turned on, the person doing the review signs it off and the work order is finished right away. Today there is nothing that stops someone from creating the customer's bill (invoice) before that review sign-off has happened. (This is the same idea we asked about last time - it was not clear then, so here it is in plainer words.)</t>
+          <t>The bill can go out straight away, before anyone reviews or approves the finished job.</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>When review is required, should the app stop anyone from billing the customer until the work order has actually been reviewed and signed off?</t>
+          <t>Should the system make someone review and approve the job first, before the customer's bill can be sent?</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>A) Yes - block billing until the review is done. No invoice can be created until someone has reviewed and signed off the work order.
-B) No - billing can happen any time; the review is just an extra step and does not hold up billing.</t>
+          <t>A) The job must be reviewed and approved before the bill can go out.
+B) It's fine to send the bill without a review.
+C) Let each shop choose for itself.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr"/>
     </row>
-    <row r="6" ht="165" customHeight="1">
+    <row r="6" ht="150" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>For a brand-new company, should "require a review" start ON or OFF?</t>
+          <t>A brand-new shop opens the app for the very first time and starts writing up repair jobs, with nothing changed yet.</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>There is a setting that makes every work order go through a review before it is finished. When a brand-new company (organization) starts using the app, we need to know what that setting should be set to out of the box, before anyone changes it.</t>
+          <t>There is a step for "someone must review a job before it's finished," and we need to decide how it should start out for a brand-new shop.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>When a new company first starts using the app, should "require a review before finishing" already be turned ON, or start OFF so they can turn it on if they want it?</t>
+          <t>When a brand-new shop first starts, should that "must review before finishing" step start turned ON or start turned OFF?</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>A) Start ON - new companies get review-required by default; they can turn it off if they don't want it.
-B) Start OFF - new companies get no review by default; they can turn it on if they want it.</t>
+          <t>A) Start turned ON.
+B) Start turned OFF.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr"/>
     </row>
-    <row r="7" ht="165" customHeight="1">
+    <row r="7" ht="150" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>What should the "are you sure you want to close this?" pop-up say and do?</t>
+          <t>Someone is part-way through a repair job that isn't finished, and they click to close it or cancel it.</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>When someone tries to close a window that they were filling in, a small pop-up can appear to check they meant to. The exact wording and the two buttons on that pop-up have not been designed yet, so we need to know how it should behave: which button just closes the little pop-up and keeps their work, and which one backs all the way out to the previous screen.</t>
+          <t>Nothing warns them - it just closes, even if the job isn't done and there is unsaved work.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>How should the confirmation pop-up work - what should the two buttons say, and what should each one do?</t>
+          <t>What should happen when someone closes or cancels a repair job that isn't finished?</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>A) One button = "stay here" (closes only the little pop-up and keeps everything they typed); the other = "leave" (backs out to the previous screen). Nothing they typed is ever thrown away just by using this pop-up.
-B) Something different - please describe the wording and what each button should do.</t>
+          <t>A) Show a pop-up message asking them to confirm before leaving.
+B) Only warn them when there is unfinished or unsaved work.
+C) No pop-up needed - just let it close.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr"/>
     </row>
-    <row r="8" ht="165" customHeight="1">
+    <row r="8" ht="150" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Where should parts that are missing a supplier sit in the receiving list?</t>
+          <t>A parts person is receiving a delivery of parts. A few of the parts don't have a supplier chosen yet, so they're bunched together in their own group.</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>On the screens where parts are received, parts that don't yet have a supplier (vendor) chosen are grouped together on their own, because someone has to pick a supplier for them before they can be received. On one receiving screen this "missing supplier" group already sits at the top; on the newer receiving screen it currently sits at the bottom. We want them to be consistent.</t>
+          <t>That "no supplier yet" group shows up at the bottom of the list on the newer receiving screen.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Should the "missing supplier" group always sit at the TOP of the list (so people deal with it first) on every receiving screen?</t>
+          <t>Where should the "no supplier yet" group appear in the receiving list?</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>A) Yes - always put the "missing supplier" group at the top on every receiving screen, so it's the first thing people see and act on.
-B) No - leave it at the bottom on the newer screen (only the older screen leads with it).</t>
+          <t>A) At the top of the list.
+B) At the bottom of the list.
+C) Mixed in with all the other parts.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr"/>
     </row>
-    <row r="9" ht="165" customHeight="1">
+    <row r="9" ht="150" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Can a work order be finished with a $0.00 selling price on a part?</t>
+          <t>A mechanic is wrapping up a repair job, but one of the parts on it still shows a price of $0.</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>When a part is added, it has a selling price (what the customer is charged for it). The newer design shows a work order being finished even when a part's selling price is still $0.00 - it shows a small note that says "$0.00 sell price, no action needed to continue" and lets the person finish. An earlier write-up said a selling price must be filled in before saving. We need to know which one is right.</t>
+          <t>The system lets them finish the job even with that $0 part price.</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Should a work order be allowed to be finished when a part still has a $0.00 selling price, or must every part have a real selling price first?</t>
+          <t>Should the system let them finish the job with a $0 part price, or stop them until a real price is entered?</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>A) Allow it - finishing with a $0.00 selling price is fine; just show the little note and let the person continue (as the newer design shows).
-B) Require a price - a part must have a real selling price before the work order can be finished (or before it can be saved).</t>
+          <t>A) Let them finish even at $0.
+B) Stop them until a price is entered.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr"/>
     </row>
-    <row r="10" ht="165" customHeight="1">
+    <row r="10" ht="150" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Should adding a part with no supplier need the "can see money figures" permission?</t>
+          <t>Someone is adding a part to a repair job, but no supplier has been chosen for that part yet.</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Some staff have permission to see money figures (costs and selling prices) and some do not. A person can add a part that has no supplier yet. We used to assume this required the "can see money figures" permission because a selling price had to be typed in - but you've since told us a selling price is NOT required here, so that reason no longer holds. We need to know whether that permission should still be required to add a part with no supplier.</t>
+          <t>Anyone who can work on the job is able to add a part like this.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Should adding a part that has no supplier yet still require the "can see money figures" permission, or should anyone who can edit the work order be able to add one?</t>
+          <t>Who should be allowed to add a part that has no supplier yet?</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>A) Yes, still require it - only people who can see money figures can add a part with no supplier.
-B) No - anyone who can edit the work order can add a part with no supplier (money figures aren't involved anymore).</t>
+          <t>A) Only people who are allowed to see prices and money figures.
+B) Anyone who can edit the repair job.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr"/>

</xml_diff>